<commit_message>
Arreglar problema datos de Atacama
</commit_message>
<xml_diff>
--- a/dataset/datos.xlsx
+++ b/dataset/datos.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regiones_Generacion" sheetId="1" r:id="R1f2ddc8a5a0b4457"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas_DS8" sheetId="2" r:id="R500722d257804437"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centros_Acopio" sheetId="3" r:id="R145f8c8adef145e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plantas_Tecnologias" sheetId="4" r:id="Rfb023debfd6a4445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tecnologias_Costos" sheetId="5" r:id="Rdaef245be9cb4cf2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costos_Transporte" sheetId="6" r:id="Ra30295314cc742fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos_Inversion" sheetId="7" r:id="R510dd3e9a79e4887"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Regiones_Generacion" sheetId="1" r:id="R9595d8fdf78c4560"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metas_DS8" sheetId="2" r:id="R076c4973da86418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Centros_Acopio" sheetId="3" r:id="R1d37b0d379114372"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Plantas_Tecnologias" sheetId="4" r:id="R63f9be522a2843cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tecnologias_Costos" sheetId="5" r:id="R720631187b7d467e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Costos_Transporte" sheetId="6" r:id="R01218b61f073475e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Supuestos_Inversion" sheetId="7" r:id="Rdc060561aa164565"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Oferta_Base" sheetId="8" r:id="R2a00ce076b5641d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -404,7 +405,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="8">
+  <x:numFmts count="9">
     <x:numFmt numFmtId="164" formatCode="General"/>
     <x:numFmt numFmtId="165" formatCode="0.0%"/>
     <x:numFmt numFmtId="166" formatCode="#,##0.0"/>
@@ -413,8 +414,9 @@
     <x:numFmt numFmtId="169" formatCode="#,##0.00"/>
     <x:numFmt numFmtId="200" formatCode="0.0"/>
     <x:numFmt numFmtId="201" formatCode="#,##0"/>
+    <x:numFmt numFmtId="202" formatCode="0.0000%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="16">
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF000000"/>
@@ -483,8 +485,33 @@
       <x:name val="Arial"/>
       <x:family val="2"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF222222"/>
+      <x:name val="Arial"/>
+      <x:family val="2"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="7">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -509,6 +536,16 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF1C3557"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF244062"/>
       </x:patternFill>
     </x:fill>
     <x:fill>
@@ -581,7 +618,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="24">
+  <x:cellXfs count="48">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0" shrinkToFit="0"/>
       <x:protection locked="1" hidden="0"/>
@@ -669,6 +706,78 @@
     </x:xf>
     <x:xf numFmtId="166" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="6" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="13" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="167" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -1866,7 +1975,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R00d83f2489db482d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R5547e8dd015b45d7"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2076,6 +2185,7 @@
     <x:col min="4" max="4" width="20" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="28" hidden="0" customWidth="1"/>
     <x:col min="6" max="10" width="18" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="24" hidden="0" customHeight="1">
@@ -2109,6 +2219,9 @@
       <x:c r="J1" s="2" t="s">
         <x:v>9</x:v>
       </x:c>
+      <x:c r="K1" s="25" t="str">
+        <x:v>Vehiculos_2024 [veh]</x:v>
+      </x:c>
     </x:row>
     <x:row r="2" ht="15" hidden="0">
       <x:c r="A2" s="3" t="s">
@@ -2121,25 +2234,34 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="D2" s="4" t="n">
-        <x:v>0.007</x:v>
-      </x:c>
-      <x:c r="E2" s="4" t="n">
-        <x:v>0.014</x:v>
-      </x:c>
-      <x:c r="F2" s="5" t="n">
-        <x:v>1078</x:v>
-      </x:c>
-      <x:c r="G2" s="5" t="n">
-        <x:v>1104.95</x:v>
-      </x:c>
-      <x:c r="H2" s="5" t="n">
-        <x:v>1132.57</x:v>
-      </x:c>
-      <x:c r="I2" s="5" t="n">
-        <x:v>1160.89</x:v>
-      </x:c>
-      <x:c r="J2" s="5" t="n">
-        <x:v>1189.91</x:v>
+        <x:v>0.006999999999999999</x:v>
+      </x:c>
+      <x:c r="E2" s="26" t="n">
+        <x:f>K2/SUM($K$2:$K$17)</x:f>
+        <x:v>0.013899087293166629</x:v>
+      </x:c>
+      <x:c r="F2" s="29" t="n">
+        <x:f>$E2*'Oferta_Base'!$B$2</x:f>
+        <x:v>2049.0034487586245</x:v>
+      </x:c>
+      <x:c r="G2" s="29" t="n">
+        <x:f>$E2*'Oferta_Base'!$B$3</x:f>
+        <x:v>2100.2285349775902</x:v>
+      </x:c>
+      <x:c r="H2" s="29" t="n">
+        <x:f>$E2*'Oferta_Base'!$B$4</x:f>
+        <x:v>2152.7342483520297</x:v>
+      </x:c>
+      <x:c r="I2" s="29" t="n">
+        <x:f>$E2*'Oferta_Base'!$B$5</x:f>
+        <x:v>2206.55260456083</x:v>
+      </x:c>
+      <x:c r="J2" s="29" t="n">
+        <x:f>$E2*'Oferta_Base'!$B$6</x:f>
+        <x:v>2261.7164196748504</x:v>
+      </x:c>
+      <x:c r="K2" s="24" t="n">
+        <x:v>91634</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="15" hidden="0">
@@ -2155,23 +2277,32 @@
       <x:c r="D3" s="7" t="n">
         <x:v>0.012</x:v>
       </x:c>
-      <x:c r="E3" s="7" t="n">
-        <x:v>0.024</x:v>
-      </x:c>
-      <x:c r="F3" s="8" t="n">
-        <x:v>1848</x:v>
-      </x:c>
-      <x:c r="G3" s="8" t="n">
-        <x:v>1894.2</x:v>
-      </x:c>
-      <x:c r="H3" s="8" t="n">
-        <x:v>1941.55</x:v>
-      </x:c>
-      <x:c r="I3" s="8" t="n">
-        <x:v>1990.09</x:v>
-      </x:c>
-      <x:c r="J3" s="8" t="n">
-        <x:v>2039.85</x:v>
+      <x:c r="E3" s="27" t="n">
+        <x:f>K3/SUM($K$2:$K$17)</x:f>
+        <x:v>0.02503789357097819</x:v>
+      </x:c>
+      <x:c r="F3" s="30" t="n">
+        <x:f>$E3*'Oferta_Base'!$B$2</x:f>
+        <x:v>3691.086270233605</x:v>
+      </x:c>
+      <x:c r="G3" s="30" t="n">
+        <x:f>$E3*'Oferta_Base'!$B$3</x:f>
+        <x:v>3783.363426989445</x:v>
+      </x:c>
+      <x:c r="H3" s="30" t="n">
+        <x:f>$E3*'Oferta_Base'!$B$4</x:f>
+        <x:v>3877.9475126641805</x:v>
+      </x:c>
+      <x:c r="I3" s="30" t="n">
+        <x:f>$E3*'Oferta_Base'!$B$5</x:f>
+        <x:v>3974.896200480784</x:v>
+      </x:c>
+      <x:c r="J3" s="30" t="n">
+        <x:f>$E3*'Oferta_Base'!$B$6</x:f>
+        <x:v>4074.268605492804</x:v>
+      </x:c>
+      <x:c r="K3" s="24" t="n">
+        <x:v>165070</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
@@ -2187,23 +2318,32 @@
       <x:c r="D4" s="4" t="n">
         <x:v>0.024</x:v>
       </x:c>
-      <x:c r="E4" s="4" t="n">
-        <x:v>0.048</x:v>
-      </x:c>
-      <x:c r="F4" s="5" t="n">
-        <x:v>3696</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="n">
-        <x:v>3788.4</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="n">
-        <x:v>3883.11</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="n">
-        <x:v>3980.19</x:v>
-      </x:c>
-      <x:c r="J4" s="5" t="n">
-        <x:v>4079.69</x:v>
+      <x:c r="E4" s="26" t="n">
+        <x:f>K4/SUM($K$2:$K$17)</x:f>
+        <x:v>0.027585670261544133</x:v>
+      </x:c>
+      <x:c r="F4" s="29" t="n">
+        <x:f>$E4*'Oferta_Base'!$B$2</x:f>
+        <x:v>4066.6795099568362</x:v>
+      </x:c>
+      <x:c r="G4" s="29" t="n">
+        <x:f>$E4*'Oferta_Base'!$B$3</x:f>
+        <x:v>4168.346497705757</x:v>
+      </x:c>
+      <x:c r="H4" s="29" t="n">
+        <x:f>$E4*'Oferta_Base'!$B$4</x:f>
+        <x:v>4272.5551601484</x:v>
+      </x:c>
+      <x:c r="I4" s="29" t="n">
+        <x:f>$E4*'Oferta_Base'!$B$5</x:f>
+        <x:v>4379.3690391521095</x:v>
+      </x:c>
+      <x:c r="J4" s="29" t="n">
+        <x:f>$E4*'Oferta_Base'!$B$6</x:f>
+        <x:v>4488.853265130912</x:v>
+      </x:c>
+      <x:c r="K4" s="24" t="n">
+        <x:v>181867</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
@@ -2219,23 +2359,32 @@
       <x:c r="D5" s="7" t="n">
         <x:v>0.025</x:v>
       </x:c>
-      <x:c r="E5" s="7" t="n">
-        <x:v>0.05</x:v>
-      </x:c>
-      <x:c r="F5" s="8" t="n">
-        <x:v>3850</x:v>
-      </x:c>
-      <x:c r="G5" s="8" t="n">
-        <x:v>3946.25</x:v>
-      </x:c>
-      <x:c r="H5" s="8" t="n">
-        <x:v>4044.91</x:v>
-      </x:c>
-      <x:c r="I5" s="8" t="n">
-        <x:v>4146.03</x:v>
-      </x:c>
-      <x:c r="J5" s="8" t="n">
-        <x:v>4249.68</x:v>
+      <x:c r="E5" s="27" t="n">
+        <x:f>K5/SUM($K$2:$K$17)</x:f>
+        <x:v>0.01626515079237114</x:v>
+      </x:c>
+      <x:c r="F5" s="30" t="n">
+        <x:f>$E5*'Oferta_Base'!$B$2</x:f>
+        <x:v>2397.8085298113533</x:v>
+      </x:c>
+      <x:c r="G5" s="30" t="n">
+        <x:f>$E5*'Oferta_Base'!$B$3</x:f>
+        <x:v>2457.753743056637</x:v>
+      </x:c>
+      <x:c r="H5" s="30" t="n">
+        <x:f>$E5*'Oferta_Base'!$B$4</x:f>
+        <x:v>2519.197586633053</x:v>
+      </x:c>
+      <x:c r="I5" s="30" t="n">
+        <x:f>$E5*'Oferta_Base'!$B$5</x:f>
+        <x:v>2582.1775262988785</x:v>
+      </x:c>
+      <x:c r="J5" s="30" t="n">
+        <x:f>$E5*'Oferta_Base'!$B$6</x:f>
+        <x:v>2646.731964456351</x:v>
+      </x:c>
+      <x:c r="K5" s="24" t="n">
+        <x:v>107233</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
@@ -2251,23 +2400,32 @@
       <x:c r="D6" s="4" t="n">
         <x:v>0.021</x:v>
       </x:c>
-      <x:c r="E6" s="4" t="n">
-        <x:v>0.042</x:v>
-      </x:c>
-      <x:c r="F6" s="5" t="n">
-        <x:v>3234</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="n">
-        <x:v>3314.85</x:v>
-      </x:c>
-      <x:c r="H6" s="5" t="n">
-        <x:v>3397.72</x:v>
-      </x:c>
-      <x:c r="I6" s="5" t="n">
-        <x:v>3482.66</x:v>
-      </x:c>
-      <x:c r="J6" s="5" t="n">
-        <x:v>3569.73</x:v>
+      <x:c r="E6" s="26" t="n">
+        <x:f>K6/SUM($K$2:$K$17)</x:f>
+        <x:v>0.0435221294965862</x:v>
+      </x:c>
+      <x:c r="F6" s="29" t="n">
+        <x:f>$E6*'Oferta_Base'!$B$2</x:f>
+        <x:v>6416.032330386738</x:v>
+      </x:c>
+      <x:c r="G6" s="29" t="n">
+        <x:f>$E6*'Oferta_Base'!$B$3</x:f>
+        <x:v>6576.433138646406</x:v>
+      </x:c>
+      <x:c r="H6" s="29" t="n">
+        <x:f>$E6*'Oferta_Base'!$B$4</x:f>
+        <x:v>6740.843967112566</x:v>
+      </x:c>
+      <x:c r="I6" s="29" t="n">
+        <x:f>$E6*'Oferta_Base'!$B$5</x:f>
+        <x:v>6909.365066290378</x:v>
+      </x:c>
+      <x:c r="J6" s="29" t="n">
+        <x:f>$E6*'Oferta_Base'!$B$6</x:f>
+        <x:v>7082.099192947638</x:v>
+      </x:c>
+      <x:c r="K6" s="24" t="n">
+        <x:v>286933</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
@@ -2283,23 +2441,32 @@
       <x:c r="D7" s="7" t="n">
         <x:v>0.047</x:v>
       </x:c>
-      <x:c r="E7" s="7" t="n">
-        <x:v>0.094</x:v>
-      </x:c>
-      <x:c r="F7" s="8" t="n">
-        <x:v>7238</x:v>
-      </x:c>
-      <x:c r="G7" s="8" t="n">
-        <x:v>7418.95</x:v>
-      </x:c>
-      <x:c r="H7" s="8" t="n">
-        <x:v>7604.42</x:v>
-      </x:c>
-      <x:c r="I7" s="8" t="n">
-        <x:v>7794.53</x:v>
-      </x:c>
-      <x:c r="J7" s="8" t="n">
-        <x:v>7989.4</x:v>
+      <x:c r="E7" s="27" t="n">
+        <x:f>K7/SUM($K$2:$K$17)</x:f>
+        <x:v>0.10608561724922329</x:v>
+      </x:c>
+      <x:c r="F7" s="30" t="n">
+        <x:f>$E7*'Oferta_Base'!$B$2</x:f>
+        <x:v>15639.141694880496</x:v>
+      </x:c>
+      <x:c r="G7" s="30" t="n">
+        <x:f>$E7*'Oferta_Base'!$B$3</x:f>
+        <x:v>16030.12023725251</x:v>
+      </x:c>
+      <x:c r="H7" s="30" t="n">
+        <x:f>$E7*'Oferta_Base'!$B$4</x:f>
+        <x:v>16430.87324318382</x:v>
+      </x:c>
+      <x:c r="I7" s="30" t="n">
+        <x:f>$E7*'Oferta_Base'!$B$5</x:f>
+        <x:v>16841.64507426341</x:v>
+      </x:c>
+      <x:c r="J7" s="30" t="n">
+        <x:f>$E7*'Oferta_Base'!$B$6</x:f>
+        <x:v>17262.686201119996</x:v>
+      </x:c>
+      <x:c r="K7" s="24" t="n">
+        <x:v>699402</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
@@ -2315,23 +2482,32 @@
       <x:c r="D8" s="4" t="n">
         <x:v>0.153</x:v>
       </x:c>
-      <x:c r="E8" s="4" t="n">
-        <x:v>0.306</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="n">
-        <x:v>23562</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="n">
-        <x:v>24151.05</x:v>
-      </x:c>
-      <x:c r="H8" s="5" t="n">
-        <x:v>24754.82</x:v>
-      </x:c>
-      <x:c r="I8" s="5" t="n">
-        <x:v>25373.7</x:v>
-      </x:c>
-      <x:c r="J8" s="5" t="n">
-        <x:v>26008.04</x:v>
+      <x:c r="E8" s="26" t="n">
+        <x:f>K8/SUM($K$2:$K$17)</x:f>
+        <x:v>0.37048513630082</x:v>
+      </x:c>
+      <x:c r="F8" s="29" t="n">
+        <x:f>$E8*'Oferta_Base'!$B$2</x:f>
+        <x:v>54616.91879346688</x:v>
+      </x:c>
+      <x:c r="G8" s="29" t="n">
+        <x:f>$E8*'Oferta_Base'!$B$3</x:f>
+        <x:v>55982.34176330355</x:v>
+      </x:c>
+      <x:c r="H8" s="29" t="n">
+        <x:f>$E8*'Oferta_Base'!$B$4</x:f>
+        <x:v>57381.90030738613</x:v>
+      </x:c>
+      <x:c r="I8" s="29" t="n">
+        <x:f>$E8*'Oferta_Base'!$B$5</x:f>
+        <x:v>58816.44781507077</x:v>
+      </x:c>
+      <x:c r="J8" s="29" t="n">
+        <x:f>$E8*'Oferta_Base'!$B$6</x:f>
+        <x:v>60286.859010447544</x:v>
+      </x:c>
+      <x:c r="K8" s="24" t="n">
+        <x:v>2442537</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
@@ -2347,23 +2523,32 @@
       <x:c r="D9" s="7" t="n">
         <x:v>0.035</x:v>
       </x:c>
-      <x:c r="E9" s="7" t="n">
-        <x:v>0.07</x:v>
-      </x:c>
-      <x:c r="F9" s="8" t="n">
-        <x:v>5390</x:v>
-      </x:c>
-      <x:c r="G9" s="8" t="n">
-        <x:v>5524.75</x:v>
-      </x:c>
-      <x:c r="H9" s="8" t="n">
-        <x:v>5662.87</x:v>
-      </x:c>
-      <x:c r="I9" s="8" t="n">
-        <x:v>5804.44</x:v>
-      </x:c>
-      <x:c r="J9" s="8" t="n">
-        <x:v>5949.55</x:v>
+      <x:c r="E9" s="27" t="n">
+        <x:f>K9/SUM($K$2:$K$17)</x:f>
+        <x:v>0.059704159396748606</x:v>
+      </x:c>
+      <x:c r="F9" s="30" t="n">
+        <x:f>$E9*'Oferta_Base'!$B$2</x:f>
+        <x:v>8801.587178268679</x:v>
+      </x:c>
+      <x:c r="G9" s="30" t="n">
+        <x:f>$E9*'Oferta_Base'!$B$3</x:f>
+        <x:v>9021.626857725396</x:v>
+      </x:c>
+      <x:c r="H9" s="30" t="n">
+        <x:f>$E9*'Oferta_Base'!$B$4</x:f>
+        <x:v>9247.16752916853</x:v>
+      </x:c>
+      <x:c r="I9" s="30" t="n">
+        <x:f>$E9*'Oferta_Base'!$B$5</x:f>
+        <x:v>9478.34671739774</x:v>
+      </x:c>
+      <x:c r="J9" s="30" t="n">
+        <x:f>$E9*'Oferta_Base'!$B$6</x:f>
+        <x:v>9715.305385332686</x:v>
+      </x:c>
+      <x:c r="K9" s="24" t="n">
+        <x:v>393618</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
@@ -2379,23 +2564,32 @@
       <x:c r="D10" s="4" t="n">
         <x:v>0.042</x:v>
       </x:c>
-      <x:c r="E10" s="4" t="n">
-        <x:v>0.084</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="n">
-        <x:v>6468</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="n">
-        <x:v>6629.7</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="n">
-        <x:v>6795.44</x:v>
-      </x:c>
-      <x:c r="I10" s="5" t="n">
-        <x:v>6965.33</x:v>
-      </x:c>
-      <x:c r="J10" s="5" t="n">
-        <x:v>7139.46</x:v>
+      <x:c r="E10" s="26" t="n">
+        <x:f>K10/SUM($K$2:$K$17)</x:f>
+        <x:v>0.0820181752628281</x:v>
+      </x:c>
+      <x:c r="F10" s="29" t="n">
+        <x:f>$E10*'Oferta_Base'!$B$2</x:f>
+        <x:v>12091.119397246119</x:v>
+      </x:c>
+      <x:c r="G10" s="29" t="n">
+        <x:f>$E10*'Oferta_Base'!$B$3</x:f>
+        <x:v>12393.397382177272</x:v>
+      </x:c>
+      <x:c r="H10" s="29" t="n">
+        <x:f>$E10*'Oferta_Base'!$B$4</x:f>
+        <x:v>12703.232316731703</x:v>
+      </x:c>
+      <x:c r="I10" s="29" t="n">
+        <x:f>$E10*'Oferta_Base'!$B$5</x:f>
+        <x:v>13020.813124649992</x:v>
+      </x:c>
+      <x:c r="J10" s="29" t="n">
+        <x:f>$E10*'Oferta_Base'!$B$6</x:f>
+        <x:v>13346.333452766243</x:v>
+      </x:c>
+      <x:c r="K10" s="24" t="n">
+        <x:v>540730</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
@@ -2411,23 +2605,32 @@
       <x:c r="D11" s="7" t="n">
         <x:v>0.016</x:v>
       </x:c>
-      <x:c r="E11" s="7" t="n">
-        <x:v>0.032</x:v>
-      </x:c>
-      <x:c r="F11" s="8" t="n">
-        <x:v>2464</x:v>
-      </x:c>
-      <x:c r="G11" s="8" t="n">
-        <x:v>2525.6</x:v>
-      </x:c>
-      <x:c r="H11" s="8" t="n">
-        <x:v>2588.74</x:v>
-      </x:c>
-      <x:c r="I11" s="8" t="n">
-        <x:v>2653.46</x:v>
-      </x:c>
-      <x:c r="J11" s="8" t="n">
-        <x:v>2719.79</x:v>
+      <x:c r="E11" s="27" t="n">
+        <x:f>K11/SUM($K$2:$K$17)</x:f>
+        <x:v>0.029125378613388805</x:v>
+      </x:c>
+      <x:c r="F11" s="30" t="n">
+        <x:f>$E11*'Oferta_Base'!$B$2</x:f>
+        <x:v>4293.663315185778</x:v>
+      </x:c>
+      <x:c r="G11" s="30" t="n">
+        <x:f>$E11*'Oferta_Base'!$B$3</x:f>
+        <x:v>4401.004898065422</x:v>
+      </x:c>
+      <x:c r="H11" s="30" t="n">
+        <x:f>$E11*'Oferta_Base'!$B$4</x:f>
+        <x:v>4511.030020517057</x:v>
+      </x:c>
+      <x:c r="I11" s="30" t="n">
+        <x:f>$E11*'Oferta_Base'!$B$5</x:f>
+        <x:v>4623.805771029983</x:v>
+      </x:c>
+      <x:c r="J11" s="30" t="n">
+        <x:f>$E11*'Oferta_Base'!$B$6</x:f>
+        <x:v>4739.400915305732</x:v>
+      </x:c>
+      <x:c r="K11" s="24" t="n">
+        <x:v>192018</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="15" hidden="0">
@@ -2443,23 +2646,32 @@
       <x:c r="D12" s="4" t="n">
         <x:v>0.042</x:v>
       </x:c>
-      <x:c r="E12" s="4" t="n">
-        <x:v>0.084</x:v>
-      </x:c>
-      <x:c r="F12" s="5" t="n">
-        <x:v>6468</x:v>
-      </x:c>
-      <x:c r="G12" s="5" t="n">
-        <x:v>6629.7</x:v>
-      </x:c>
-      <x:c r="H12" s="5" t="n">
-        <x:v>6795.44</x:v>
-      </x:c>
-      <x:c r="I12" s="5" t="n">
-        <x:v>6965.33</x:v>
-      </x:c>
-      <x:c r="J12" s="5" t="n">
-        <x:v>7139.46</x:v>
+      <x:c r="E12" s="26" t="n">
+        <x:f>K12/SUM($K$2:$K$17)</x:f>
+        <x:v>0.08251841742068287</x:v>
+      </x:c>
+      <x:c r="F12" s="29" t="n">
+        <x:f>$E12*'Oferta_Base'!$B$2</x:f>
+        <x:v>12164.86509615707</x:v>
+      </x:c>
+      <x:c r="G12" s="29" t="n">
+        <x:f>$E12*'Oferta_Base'!$B$3</x:f>
+        <x:v>12468.986723560996</x:v>
+      </x:c>
+      <x:c r="H12" s="29" t="n">
+        <x:f>$E12*'Oferta_Base'!$B$4</x:f>
+        <x:v>12780.71139165002</x:v>
+      </x:c>
+      <x:c r="I12" s="29" t="n">
+        <x:f>$E12*'Oferta_Base'!$B$5</x:f>
+        <x:v>13100.229176441268</x:v>
+      </x:c>
+      <x:c r="J12" s="29" t="n">
+        <x:f>$E12*'Oferta_Base'!$B$6</x:f>
+        <x:v>13427.734905852298</x:v>
+      </x:c>
+      <x:c r="K12" s="24" t="n">
+        <x:v>544028</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
@@ -2473,25 +2685,34 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="D13" s="7" t="n">
-        <x:v>0.026</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="n">
-        <x:v>0.052</x:v>
-      </x:c>
-      <x:c r="F13" s="8" t="n">
-        <x:v>4004</x:v>
-      </x:c>
-      <x:c r="G13" s="8" t="n">
-        <x:v>4104.1</x:v>
-      </x:c>
-      <x:c r="H13" s="8" t="n">
-        <x:v>4206.7</x:v>
-      </x:c>
-      <x:c r="I13" s="8" t="n">
-        <x:v>4311.87</x:v>
-      </x:c>
-      <x:c r="J13" s="8" t="n">
-        <x:v>4419.67</x:v>
+        <x:v>0.026000000000000002</x:v>
+      </x:c>
+      <x:c r="E13" s="27" t="n">
+        <x:f>K13/SUM($K$2:$K$17)</x:f>
+        <x:v>0.0483370740262835</x:v>
+      </x:c>
+      <x:c r="F13" s="30" t="n">
+        <x:f>$E13*'Oferta_Base'!$B$2</x:f>
+        <x:v>7125.851452954713</x:v>
+      </x:c>
+      <x:c r="G13" s="30" t="n">
+        <x:f>$E13*'Oferta_Base'!$B$3</x:f>
+        <x:v>7303.997739278581</x:v>
+      </x:c>
+      <x:c r="H13" s="30" t="n">
+        <x:f>$E13*'Oferta_Base'!$B$4</x:f>
+        <x:v>7486.597682760545</x:v>
+      </x:c>
+      <x:c r="I13" s="30" t="n">
+        <x:f>$E13*'Oferta_Base'!$B$5</x:f>
+        <x:v>7673.762624829556</x:v>
+      </x:c>
+      <x:c r="J13" s="30" t="n">
+        <x:f>$E13*'Oferta_Base'!$B$6</x:f>
+        <x:v>7865.606690450295</x:v>
+      </x:c>
+      <x:c r="K13" s="24" t="n">
+        <x:v>318677</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
@@ -2505,25 +2726,34 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="D14" s="4" t="n">
-        <x:v>0.011</x:v>
-      </x:c>
-      <x:c r="E14" s="4" t="n">
-        <x:v>0.022</x:v>
-      </x:c>
-      <x:c r="F14" s="5" t="n">
-        <x:v>1694</x:v>
-      </x:c>
-      <x:c r="G14" s="5" t="n">
-        <x:v>1736.35</x:v>
-      </x:c>
-      <x:c r="H14" s="5" t="n">
-        <x:v>1779.76</x:v>
-      </x:c>
-      <x:c r="I14" s="5" t="n">
-        <x:v>1824.25</x:v>
-      </x:c>
-      <x:c r="J14" s="5" t="n">
-        <x:v>1869.86</x:v>
+        <x:v>0.011000000000000001</x:v>
+      </x:c>
+      <x:c r="E14" s="26" t="n">
+        <x:f>K14/SUM($K$2:$K$17)</x:f>
+        <x:v>0.022305976801687052</x:v>
+      </x:c>
+      <x:c r="F14" s="29" t="n">
+        <x:f>$E14*'Oferta_Base'!$B$2</x:f>
+        <x:v>3288.347100104705</x:v>
+      </x:c>
+      <x:c r="G14" s="29" t="n">
+        <x:f>$E14*'Oferta_Base'!$B$3</x:f>
+        <x:v>3370.555777607323</x:v>
+      </x:c>
+      <x:c r="H14" s="29" t="n">
+        <x:f>$E14*'Oferta_Base'!$B$4</x:f>
+        <x:v>3454.8196720475053</x:v>
+      </x:c>
+      <x:c r="I14" s="29" t="n">
+        <x:f>$E14*'Oferta_Base'!$B$5</x:f>
+        <x:v>3541.1901638486925</x:v>
+      </x:c>
+      <x:c r="J14" s="29" t="n">
+        <x:f>$E14*'Oferta_Base'!$B$6</x:f>
+        <x:v>3629.7199179449094</x:v>
+      </x:c>
+      <x:c r="K14" s="24" t="n">
+        <x:v>147059</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0">
@@ -2537,25 +2767,34 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="D15" s="7" t="n">
-        <x:v>0.027</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="n">
-        <x:v>0.054</x:v>
-      </x:c>
-      <x:c r="F15" s="8" t="n">
-        <x:v>4158</x:v>
-      </x:c>
-      <x:c r="G15" s="8" t="n">
-        <x:v>4261.95</x:v>
-      </x:c>
-      <x:c r="H15" s="8" t="n">
-        <x:v>4368.5</x:v>
-      </x:c>
-      <x:c r="I15" s="8" t="n">
-        <x:v>4477.71</x:v>
-      </x:c>
-      <x:c r="J15" s="8" t="n">
-        <x:v>4589.65</x:v>
+        <x:v>0.027000000000000003</x:v>
+      </x:c>
+      <x:c r="E15" s="27" t="n">
+        <x:f>K15/SUM($K$2:$K$17)</x:f>
+        <x:v>0.050365800181925546</x:v>
+      </x:c>
+      <x:c r="F15" s="30" t="n">
+        <x:f>$E15*'Oferta_Base'!$B$2</x:f>
+        <x:v>7424.926262819464</x:v>
+      </x:c>
+      <x:c r="G15" s="30" t="n">
+        <x:f>$E15*'Oferta_Base'!$B$3</x:f>
+        <x:v>7610.54941938995</x:v>
+      </x:c>
+      <x:c r="H15" s="30" t="n">
+        <x:f>$E15*'Oferta_Base'!$B$4</x:f>
+        <x:v>7800.813154874699</x:v>
+      </x:c>
+      <x:c r="I15" s="30" t="n">
+        <x:f>$E15*'Oferta_Base'!$B$5</x:f>
+        <x:v>7995.8334837465645</x:v>
+      </x:c>
+      <x:c r="J15" s="30" t="n">
+        <x:f>$E15*'Oferta_Base'!$B$6</x:f>
+        <x:v>8195.729320840228</x:v>
+      </x:c>
+      <x:c r="K15" s="24" t="n">
+        <x:v>332052</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0">
@@ -2571,23 +2810,32 @@
       <x:c r="D16" s="4" t="n">
         <x:v>0.005</x:v>
       </x:c>
-      <x:c r="E16" s="4" t="n">
-        <x:v>0.01</x:v>
-      </x:c>
-      <x:c r="F16" s="5" t="n">
-        <x:v>770</x:v>
-      </x:c>
-      <x:c r="G16" s="5" t="n">
-        <x:v>789.25</x:v>
-      </x:c>
-      <x:c r="H16" s="5" t="n">
-        <x:v>808.98</x:v>
-      </x:c>
-      <x:c r="I16" s="5" t="n">
-        <x:v>829.21</x:v>
-      </x:c>
-      <x:c r="J16" s="5" t="n">
-        <x:v>849.94</x:v>
+      <x:c r="E16" s="26" t="n">
+        <x:f>K16/SUM($K$2:$K$17)</x:f>
+        <x:v>0.008791854516596649</x:v>
+      </x:c>
+      <x:c r="F16" s="29" t="n">
+        <x:f>$E16*'Oferta_Base'!$B$2</x:f>
+        <x:v>1296.095192836678</x:v>
+      </x:c>
+      <x:c r="G16" s="29" t="n">
+        <x:f>$E16*'Oferta_Base'!$B$3</x:f>
+        <x:v>1328.497572657595</x:v>
+      </x:c>
+      <x:c r="H16" s="29" t="n">
+        <x:f>$E16*'Oferta_Base'!$B$4</x:f>
+        <x:v>1361.7100119740346</x:v>
+      </x:c>
+      <x:c r="I16" s="29" t="n">
+        <x:f>$E16*'Oferta_Base'!$B$5</x:f>
+        <x:v>1395.7527622733853</x:v>
+      </x:c>
+      <x:c r="J16" s="29" t="n">
+        <x:f>$E16*'Oferta_Base'!$B$6</x:f>
+        <x:v>1430.6465813302198</x:v>
+      </x:c>
+      <x:c r="K16" s="24" t="n">
+        <x:v>57963</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0">
@@ -2601,25 +2849,34 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="D17" s="7" t="n">
-        <x:v>0.007</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="n">
-        <x:v>0.014</x:v>
-      </x:c>
-      <x:c r="F17" s="8" t="n">
-        <x:v>1078</x:v>
-      </x:c>
-      <x:c r="G17" s="8" t="n">
-        <x:v>1104.95</x:v>
-      </x:c>
-      <x:c r="H17" s="8" t="n">
-        <x:v>1132.57</x:v>
-      </x:c>
-      <x:c r="I17" s="8" t="n">
-        <x:v>1160.89</x:v>
-      </x:c>
-      <x:c r="J17" s="8" t="n">
-        <x:v>1189.91</x:v>
+        <x:v>0.006999999999999999</x:v>
+      </x:c>
+      <x:c r="E17" s="27" t="n">
+        <x:f>K17/SUM($K$2:$K$17)</x:f>
+        <x:v>0.01395247881516932</x:v>
+      </x:c>
+      <x:c r="F17" s="30" t="n">
+        <x:f>$E17*'Oferta_Base'!$B$2</x:f>
+        <x:v>2056.874426932261</x:v>
+      </x:c>
+      <x:c r="G17" s="30" t="n">
+        <x:f>$E17*'Oferta_Base'!$B$3</x:f>
+        <x:v>2108.2962876055676</x:v>
+      </x:c>
+      <x:c r="H17" s="30" t="n">
+        <x:f>$E17*'Oferta_Base'!$B$4</x:f>
+        <x:v>2161.0036947957065</x:v>
+      </x:c>
+      <x:c r="I17" s="30" t="n">
+        <x:f>$E17*'Oferta_Base'!$B$5</x:f>
+        <x:v>2215.0287871655987</x:v>
+      </x:c>
+      <x:c r="J17" s="30" t="n">
+        <x:f>$E17*'Oferta_Base'!$B$6</x:f>
+        <x:v>2270.4045068447385</x:v>
+      </x:c>
+      <x:c r="K17" s="24" t="n">
+        <x:v>91986</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0">
@@ -2636,34 +2893,38 @@
         <x:f aca="0">SUM(D2:D17)</x:f>
         <x:v>0.5000000000000001</x:v>
       </x:c>
-      <x:c r="E18" s="10" t="n">
+      <x:c r="E18" s="28" t="n">
         <x:f aca="0">SUM(E2:E17)</x:f>
-        <x:v>1.0000000000000002</x:v>
-      </x:c>
-      <x:c r="F18" s="11" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="F18" s="31" t="n">
         <x:f aca="0">SUM(F2:F17)</x:f>
-        <x:v>77000</x:v>
-      </x:c>
-      <x:c r="G18" s="11" t="n">
+        <x:v>147420</x:v>
+      </x:c>
+      <x:c r="G18" s="31" t="n">
         <x:f aca="0">SUM(G2:G17)</x:f>
-        <x:v>78925</x:v>
-      </x:c>
-      <x:c r="H18" s="11" t="n">
+        <x:v>151105.5</x:v>
+      </x:c>
+      <x:c r="H18" s="31" t="n">
         <x:f aca="0">SUM(H2:H17)</x:f>
-        <x:v>80898.09999999999</x:v>
-      </x:c>
-      <x:c r="I18" s="11" t="n">
+        <x:v>154883.13749999998</x:v>
+      </x:c>
+      <x:c r="I18" s="31" t="n">
         <x:f aca="0">SUM(I2:I17)</x:f>
-        <x:v>82920.58</x:v>
-      </x:c>
-      <x:c r="J18" s="11" t="n">
+        <x:v>158755.21593749992</x:v>
+      </x:c>
+      <x:c r="J18" s="31" t="n">
         <x:f aca="0">SUM(J2:J17)</x:f>
-        <x:v>84993.59000000001</x:v>
+        <x:v>162724.09633593744</x:v>
+      </x:c>
+      <x:c r="K18" s="24" t="n">
+        <x:f>SUM(K2:K17)</x:f>
+        <x:v>6592807</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c7b7c612fab4c51"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R85d89c99301b4670"/>
 </x:worksheet>
 </file>
 
@@ -8304,4 +8565,351 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="28" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="3" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="31" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="20" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="13" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="69" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="36" customHeight="1">
+      <x:c r="A1" s="37" t="str">
+        <x:v>Anio_t</x:v>
+      </x:c>
+      <x:c r="B1" s="37" t="str">
+        <x:v>Oferta_Nacional_G [ton]</x:v>
+      </x:c>
+      <x:c r="C1" s="37" t="str">
+        <x:v>Participacion_Valora_theta [-]</x:v>
+      </x:c>
+      <x:c r="D1" s="37" t="str">
+        <x:v>Base_Metas_B [ton]</x:v>
+      </x:c>
+      <x:c r="E1" s="32"/>
+      <x:c r="F1" s="37" t="str">
+        <x:v>Parametro</x:v>
+      </x:c>
+      <x:c r="G1" s="37" t="str">
+        <x:v>Valor</x:v>
+      </x:c>
+      <x:c r="H1" s="37" t="str">
+        <x:v>Unidad</x:v>
+      </x:c>
+      <x:c r="I1" s="37" t="str">
+        <x:v>Origen / criterio</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" ht="23" customHeight="1">
+      <x:c r="A2" s="43" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="B2" s="44" t="n">
+        <x:f>$G$2*$G$3*(1+$G$5)^(A2-$G$6)</x:f>
+        <x:v>147420</x:v>
+      </x:c>
+      <x:c r="C2" s="45" t="n">
+        <x:f>$G$4</x:f>
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="D2" s="44" t="n">
+        <x:f>B2*C2</x:f>
+        <x:v>76658.40000000001</x:v>
+      </x:c>
+      <x:c r="E2" s="32"/>
+      <x:c r="F2" s="32" t="str">
+        <x:v>NFU de referencia 2025</x:v>
+      </x:c>
+      <x:c r="G2" s="40" t="n">
+        <x:v>189000</x:v>
+      </x:c>
+      <x:c r="H2" s="32" t="str">
+        <x:v>ton</x:v>
+      </x:c>
+      <x:c r="I2" s="46" t="str">
+        <x:v>datos hasta ahora.xlsx: Generacion!B1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="23" customHeight="1">
+      <x:c r="A3" s="43" t="n">
+        <x:v>2027</x:v>
+      </x:c>
+      <x:c r="B3" s="44" t="n">
+        <x:f>$G$2*$G$3*(1+$G$5)^(A3-$G$6)</x:f>
+        <x:v>151105.5</x:v>
+      </x:c>
+      <x:c r="C3" s="45" t="n">
+        <x:f>$G$4</x:f>
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="D3" s="44" t="n">
+        <x:f>B3*C3</x:f>
+        <x:v>78574.86</x:v>
+      </x:c>
+      <x:c r="E3" s="32"/>
+      <x:c r="F3" s="32" t="str">
+        <x:v>Fracción de categoría A</x:v>
+      </x:c>
+      <x:c r="G3" s="41" t="n">
+        <x:v>0.78</x:v>
+      </x:c>
+      <x:c r="H3" s="32" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="I3" s="46" t="str">
+        <x:v>datos hasta ahora.xlsx: Generacion!B2</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="23" customHeight="1">
+      <x:c r="A4" s="43" t="n">
+        <x:v>2028</x:v>
+      </x:c>
+      <x:c r="B4" s="44" t="n">
+        <x:f>$G$2*$G$3*(1+$G$5)^(A4-$G$6)</x:f>
+        <x:v>154883.13749999998</x:v>
+      </x:c>
+      <x:c r="C4" s="45" t="n">
+        <x:f>$G$4</x:f>
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="D4" s="44" t="n">
+        <x:f>B4*C4</x:f>
+        <x:v>80539.2315</x:v>
+      </x:c>
+      <x:c r="E4" s="32"/>
+      <x:c r="F4" s="32" t="str">
+        <x:v>Participación de Valora Más</x:v>
+      </x:c>
+      <x:c r="G4" s="41" t="n">
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="H4" s="32" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="I4" s="46" t="str">
+        <x:v>datos hasta ahora.xlsx: Generacion!B3</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="23" customHeight="1">
+      <x:c r="A5" s="43" t="n">
+        <x:v>2029</x:v>
+      </x:c>
+      <x:c r="B5" s="44" t="n">
+        <x:f>$G$2*$G$3*(1+$G$5)^(A5-$G$6)</x:f>
+        <x:v>158755.21593749995</x:v>
+      </x:c>
+      <x:c r="C5" s="45" t="n">
+        <x:f>$G$4</x:f>
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="D5" s="44" t="n">
+        <x:f>B5*C5</x:f>
+        <x:v>82552.71228749998</x:v>
+      </x:c>
+      <x:c r="E5" s="32"/>
+      <x:c r="F5" s="32" t="str">
+        <x:v>Crecimiento anual</x:v>
+      </x:c>
+      <x:c r="G5" s="41" t="n">
+        <x:v>0.025</x:v>
+      </x:c>
+      <x:c r="H5" s="32" t="str">
+        <x:v>fracción</x:v>
+      </x:c>
+      <x:c r="I5" s="46" t="str">
+        <x:v>datos hasta ahora.xlsx: Generacion!B4</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="23" customHeight="1">
+      <x:c r="A6" s="43" t="n">
+        <x:v>2030</x:v>
+      </x:c>
+      <x:c r="B6" s="44" t="n">
+        <x:f>$G$2*$G$3*(1+$G$5)^(A6-$G$6)</x:f>
+        <x:v>162724.09633593744</x:v>
+      </x:c>
+      <x:c r="C6" s="45" t="n">
+        <x:f>$G$4</x:f>
+        <x:v>0.52</x:v>
+      </x:c>
+      <x:c r="D6" s="44" t="n">
+        <x:f>B6*C6</x:f>
+        <x:v>84616.53009468748</x:v>
+      </x:c>
+      <x:c r="E6" s="32"/>
+      <x:c r="F6" s="32" t="str">
+        <x:v>Primer año del modelo</x:v>
+      </x:c>
+      <x:c r="G6" s="42" t="n">
+        <x:v>2026</x:v>
+      </x:c>
+      <x:c r="H6" s="32" t="str">
+        <x:v>año</x:v>
+      </x:c>
+      <x:c r="I6" s="46" t="str">
+        <x:v>Primer período de Metas_DS8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="32"/>
+      <x:c r="B7" s="32"/>
+      <x:c r="C7" s="32"/>
+      <x:c r="D7" s="32"/>
+      <x:c r="E7" s="32"/>
+      <x:c r="F7" s="32"/>
+      <x:c r="G7" s="32"/>
+      <x:c r="H7" s="32"/>
+      <x:c r="I7" s="46"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="32"/>
+      <x:c r="B8" s="32"/>
+      <x:c r="C8" s="32"/>
+      <x:c r="D8" s="32"/>
+      <x:c r="E8" s="32"/>
+      <x:c r="F8" s="47" t="str">
+        <x:v>Criterio</x:v>
+      </x:c>
+      <x:c r="G8" s="32"/>
+      <x:c r="H8" s="32"/>
+      <x:c r="I8" s="46"/>
+    </x:row>
+    <x:row r="9" ht="23" customHeight="1">
+      <x:c r="A9" s="32"/>
+      <x:c r="B9" s="32"/>
+      <x:c r="C9" s="32"/>
+      <x:c r="D9" s="32"/>
+      <x:c r="E9" s="32"/>
+      <x:c r="F9" s="32" t="str">
+        <x:v>Oferta regional</x:v>
+      </x:c>
+      <x:c r="G9" s="32" t="str">
+        <x:v>g_rt = p_r G_t</x:v>
+      </x:c>
+      <x:c r="H9" s="32"/>
+      <x:c r="I9" s="46" t="str">
+        <x:v>Oferta potencial contratable; no se reserva el 52% por región.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="23" customHeight="1">
+      <x:c r="A10" s="32"/>
+      <x:c r="B10" s="32"/>
+      <x:c r="C10" s="32"/>
+      <x:c r="D10" s="32"/>
+      <x:c r="E10" s="32"/>
+      <x:c r="F10" s="32" t="str">
+        <x:v>Base de metas</x:v>
+      </x:c>
+      <x:c r="G10" s="32" t="str">
+        <x:v>B_t = theta G_t</x:v>
+      </x:c>
+      <x:c r="H10" s="32"/>
+      <x:c r="I10" s="46" t="str">
+        <x:v>Aproximación de ventas previas ajustadas por desgaste.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="23" customHeight="1">
+      <x:c r="A11" s="32"/>
+      <x:c r="B11" s="32"/>
+      <x:c r="C11" s="32"/>
+      <x:c r="D11" s="32"/>
+      <x:c r="E11" s="32"/>
+      <x:c r="F11" s="32" t="str">
+        <x:v>Desgaste</x:v>
+      </x:c>
+      <x:c r="G11" s="32" t="str">
+        <x:v>Ya incluido</x:v>
+      </x:c>
+      <x:c r="H11" s="32"/>
+      <x:c r="I11" s="46" t="str">
+        <x:v>No volver a multiplicar por 0,84.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="23" customHeight="1">
+      <x:c r="A12" s="32"/>
+      <x:c r="B12" s="32"/>
+      <x:c r="C12" s="32"/>
+      <x:c r="D12" s="32"/>
+      <x:c r="E12" s="32"/>
+      <x:c r="F12" s="32" t="str">
+        <x:v>Datos operativos</x:v>
+      </x:c>
+      <x:c r="G12" s="32" t="str">
+        <x:v>Prueba</x:v>
+      </x:c>
+      <x:c r="H12" s="32"/>
+      <x:c r="I12" s="46" t="str">
+        <x:v>Capacidades y costos conservados de la instancia anterior.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="23" customHeight="1">
+      <x:c r="A13" s="32"/>
+      <x:c r="B13" s="32"/>
+      <x:c r="C13" s="32"/>
+      <x:c r="D13" s="32"/>
+      <x:c r="E13" s="32"/>
+      <x:c r="F13" s="32" t="str">
+        <x:v>Acceso a oferta</x:v>
+      </x:c>
+      <x:c r="G13" s="32" t="str">
+        <x:v>Supuesto</x:v>
+      </x:c>
+      <x:c r="H13" s="32"/>
+      <x:c r="I13" s="46" t="str">
+        <x:v>No se modelan otros sistemas ni residuos comprometidos.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="23" customHeight="1">
+      <x:c r="A14" s="32"/>
+      <x:c r="B14" s="32"/>
+      <x:c r="C14" s="32"/>
+      <x:c r="D14" s="32"/>
+      <x:c r="E14" s="32"/>
+      <x:c r="F14" s="32"/>
+      <x:c r="G14" s="32"/>
+      <x:c r="H14" s="32"/>
+      <x:c r="I14" s="46"/>
+    </x:row>
+    <x:row r="15" ht="23" customHeight="1">
+      <x:c r="A15" s="32"/>
+      <x:c r="B15" s="32"/>
+      <x:c r="C15" s="32"/>
+      <x:c r="D15" s="32"/>
+      <x:c r="E15" s="32"/>
+      <x:c r="F15" s="32" t="str">
+        <x:v>Referencia temporal</x:v>
+      </x:c>
+      <x:c r="G15" s="32"/>
+      <x:c r="H15" s="32"/>
+      <x:c r="I15" s="46" t="str">
+        <x:v>NFU 2025 se usa como proxy de oferta del primer año, 2026.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="23" customHeight="1">
+      <x:c r="A16" s="32"/>
+      <x:c r="B16" s="32"/>
+      <x:c r="C16" s="32"/>
+      <x:c r="D16" s="32"/>
+      <x:c r="E16" s="32"/>
+      <x:c r="F16" s="32" t="str">
+        <x:v>Reparto regional</x:v>
+      </x:c>
+      <x:c r="G16" s="32"/>
+      <x:c r="H16" s="32"/>
+      <x:c r="I16" s="46" t="str">
+        <x:v>Regiones_Generacion: vehículos de 2024 del archivo recibido.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>